<commit_message>
Add Stripe careers parser with static HTML table parsing
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Career Links.xlsx
+++ b/Career Links.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="3" max="3"/>
@@ -773,6 +773,23 @@
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://stripe.com/jobs/search?query=software&amp;office_locations=North+America--Atlanta&amp;office_locations=North+America--Chicago&amp;office_locations=North+America--New+York&amp;office_locations=North+America--San+Francisco+Bridge+HQ&amp;office_locations=North+America--Seattle&amp;office_locations=North+America--South+San+Francisco&amp;office_locations=North+America--Washington+DC</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Working</t>
         </is>

</xml_diff>

<commit_message>
Extra parsers and scheduling and report
</commit_message>
<xml_diff>
--- a/Career Links.xlsx
+++ b/Career Links.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="3" max="3"/>
@@ -790,6 +790,108 @@
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://careers.walmart.com/us/en/results?searchQuery=software%20engineering%20and%20architecture%20&amp;careerareas=Technology</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Autodesk</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://autodesk.wd1.myworkdayjobs.com/Ext?q=software&amp;locationCountry=bc33aa3152ec42d4995f4791a106ed09</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Zillow</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://zillow.wd5.myworkdayjobs.com/Zillow_Group_External?q=software</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DocuSign</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://careers.docusign.com/jobs?keywords=software&amp;sortBy=posted_date&amp;page=1&amp;descending=true</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Qualtrics</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://www.qualtrics.com/careers/us/en/search-results?m=3&amp;keywords=software</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://intel.wd1.myworkdayjobs.com/External?q=software</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
         <is>
           <t>Working</t>
         </is>

</xml_diff>

<commit_message>
Zoom cloudfare crowdstrike waymo chime
</commit_message>
<xml_diff>
--- a/Career Links.xlsx
+++ b/Career Links.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="3" max="3"/>
@@ -943,6 +943,108 @@
         </is>
       </c>
       <c r="C27" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Wells Fargo</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://www.wellsfargojobs.com/en/jobs/?search=software&amp;country=United+States+of+America</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Waymo</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://careers.withwaymo.com/jobs/search?page=1&amp;country_codes%5B%5D=US&amp;query=software</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Chime</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://careers.chime.com/en/jobs/?keyword=software&amp;pagesize=20</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>https://careers.zoom.us/jobs/search?page=1&amp;country_codes%5B%5D=US&amp;query=software</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>https://www.cloudflare.com/careers/jobs/?title=software</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>CrowdStrike</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>https://crowdstrike.wd5.myworkdayjobs.com/crowdstrikecareers?q=software&amp;locationCountry=bc33aa3152ec42d4995f4791a106ed09</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
         <is>
           <t>Working</t>
         </is>

</xml_diff>